<commit_message>
Variables added to apis packages
</commit_message>
<xml_diff>
--- a/package_restful_booker_herokuapp/test_excel_ddt/testfile.xlsx
+++ b/package_restful_booker_herokuapp/test_excel_ddt/testfile.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -520,36 +520,36 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>2534</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Miranda</t>
+          <t>Brian</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Lara</t>
+          <t>Farrell</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>9500</v>
+        <v>2500</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
       <c r="F2" s="1" t="n">
-        <v>44621</v>
+        <v>45206</v>
       </c>
       <c r="G2" s="1" t="n">
-        <v>44649</v>
+        <v>45230</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>blue</t>
+          <t>purpose</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>{"bookingid":12,"booking":{"firstname":"Miranda","lastname":"Lara","totalprice":9500,"depositpaid":false,"bookingdates":{"checkin":"2022-03-01","checkout":"2022-03-29"},"additionalneeds":"blue"}}</t>
+          <t>{"bookingid":2534,"booking":{"firstname":"Brian","lastname":"Farrell","totalprice":2500,"depositpaid":true,"bookingdates":{"checkin":"2023-10-07","checkout":"2023-10-31"},"additionalneeds":"purpose"}}</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -569,63 +569,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2022-03-13 21:34:38.872</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Sarah</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Alexander</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>4998</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>True</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>44632</v>
-      </c>
-      <c r="G3" s="1" t="n">
-        <v>44642</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>because</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>{"bookingid":13,"booking":{"firstname":"Sarah","lastname":"Alexander","totalprice":4998,"depositpaid":true,"bookingdates":{"checkin":"2022-03-12","checkout":"2022-03-22"},"additionalneeds":"because"}}</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>&lt;Response [200]&gt;</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2022-03-13 21:34:56.634</t>
+          <t>2023-10-21 19:16:49.945</t>
         </is>
       </c>
     </row>
@@ -640,7 +584,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -704,6 +648,116 @@
         </is>
       </c>
       <c r="D3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>bd76c0068e441f6</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>012c183bd8d0c31</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>f66356e38cd16e0</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>981c02e3e595c39</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>admin</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>password123</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ce497f95a4e2fd6</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>200</t>
         </is>
@@ -720,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -844,6 +898,130 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>2022-03-13 21:34:48.381</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1902</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>['Martha']</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>['Sherman']</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>[5809]</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>[False]</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>['2023-10-15']</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>['2023-11-18']</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>['report']</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>{"firstname":"Martha","lastname":"Sherman","totalprice":5809,"depositpaid":false,"bookingdates":{"checkin":"2023-10-15","checkout":"2023-11-18"},"additionalneeds":"report"}</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>&lt;Response [200]&gt;</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2023-10-21 19:15:43.201</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2534</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>['Krystal']</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>['Jones']</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>[4206]</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>[True]</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>['2023-10-01']</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>['2023-11-04']</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>['whole']</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>{"firstname":"Krystal","lastname":"Jones","totalprice":4206,"depositpaid":true,"bookingdates":{"checkin":"2023-10-01","checkout":"2023-11-04"},"additionalneeds":"whole"}</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>&lt;Response [200]&gt;</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2023-10-21 19:16:55.901</t>
         </is>
       </c>
     </row>
@@ -858,7 +1036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -932,6 +1110,80 @@
       <c r="L2" t="inlineStr">
         <is>
           <t>2022-03-13 21:34:50.261</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1902</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>['Frank']</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>['Craig']</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>{"firstname":"Frank","lastname":"Craig","totalprice":5809,"depositpaid":false,"bookingdates":{"checkin":"2023-10-15","checkout":"2023-11-18"},"additionalneeds":"report"}</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>&lt;Response [200]&gt;</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2023-10-21 19:15:44.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2534</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>['Andrew']</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>['Nguyen']</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>{"firstname":"Andrew","lastname":"Nguyen","totalprice":4206,"depositpaid":true,"bookingdates":{"checkin":"2023-10-01","checkout":"2023-11-04"},"additionalneeds":"whole"}</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>&lt;Response [200]&gt;</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2023-10-21 19:16:57.215</t>
         </is>
       </c>
     </row>

</xml_diff>